<commit_message>
latest results based on simulated data uploaded
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Table_2/g_output/D6_Table_2_caratterizzazione_coorte_sottopopolazione_CAP_DPP4i.xlsx
+++ b/i_test/test_D6_Table_2/g_output/D6_Table_2_caratterizzazione_coorte_sottopopolazione_CAP_DPP4i.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -518,307 +518,477 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>589</t>
+          <t>559</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>582</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>549</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>606</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>588</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>544</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>559</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>528</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>556</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>555</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>579</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>590</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>500</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BMI pregravidico basso (&lt;18,5), n (%)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>175 (29,7%)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>145 (26,7%)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>151 (27,0%)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>140 (26,5%)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>144 (25,9%)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>141 (25,4%)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>160 (27,6%)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>166 (28,1%)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>155 (31,0%)</t>
+          <t>Età alla data indice,</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BMI pregravidico medio (18,5-24,9), n (%)</t>
+          <t xml:space="preserve">  mediana (Q1 - Q3)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>190 (32,3%)</t>
+          <t>50 (40 - 61)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>185 (34,0%)</t>
+          <t>51 (41 - 60)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>194 (34,7%)</t>
+          <t>51 (41 - 62)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>181 (34,3%)</t>
+          <t>50 (42 - 60)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>198 (35,6%)</t>
+          <t>49 (40 - 59)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>197 (35,5%)</t>
+          <t>50 (42 - 59)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>190 (32,8%)</t>
+          <t>49 (40 - 61)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>204 (34,6%)</t>
+          <t>52 (42 - 61)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>159 (31,8%)</t>
+          <t>51 (40 - 60)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BMI pregravidico alto (&gt;24,9), n (%)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>224 (38,0%)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>214 (39,3%)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>214 (38,3%)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>207 (39,2%)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>214 (38,5%)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>217 (39,1%)</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>229 (39,6%)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>220 (37,3%)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>186 (37,2%)</t>
+          <t>Classi età alla data indice</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Diabete gestazionale, n (%)</t>
+          <t xml:space="preserve">  18-44, n (%)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>157 (26,7%)</t>
+          <t>206 (36,9%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>146 (26,8%)</t>
+          <t>197 (33,8%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>146 (26,1%)</t>
+          <t>173 (33,1%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>150 (28,4%)</t>
+          <t>176 (33,1%)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>173 (31,1%)</t>
+          <t>200 (36,4%)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>138 (24,9%)</t>
+          <t>178 (34,3%)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>174 (30,1%)</t>
+          <t>214 (35,3%)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>181 (30,7%)</t>
+          <t>195 (33,2%)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>133 (26,6%)</t>
+          <t>191 (35,1%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">  45-64, n (%)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>262 (46,9%)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>290 (49,8%)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>248 (47,5%)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>260 (49,0%)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>273 (49,7%)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>262 (50,5%)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>279 (46,0%)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>286 (48,6%)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>263 (48,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BMI pregravidico basso (&lt;18,5), n (%)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>92 (16,5%)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100 (17,2%)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>97 (18,6%)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>90 (16,9%)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>78 (14,2%)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>88 (17,0%)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>106 (17,5%)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>118 (20,1%)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>83 (15,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BMI pregravidico medio (18,5-24,9), n (%)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>59 (10,6%)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>71 (12,2%)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>56 (10,7%)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>53 (10,0%)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>61 (11,1%)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>63 (12,1%)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>62 (10,2%)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>57 (9,7%)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>55 (10,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BMI pregravidico alto (&gt;24,9), n (%)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>408 (73,0%)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>411 (70,6%)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>369 (70,7%)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>388 (73,1%)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>410 (74,7%)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>368 (70,9%)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>438 (72,3%)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>413 (70,2%)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>406 (74,6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Diabete gestazionale, n (%)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>342 (61,2%)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>356 (61,2%)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>325 (62,3%)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>336 (63,3%)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>331 (60,3%)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>316 (60,9%)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>389 (64,2%)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>369 (62,8%)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>333 (61,2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Diabete pregravidico, n (%)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>443 (75,2%)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>380 (69,9%)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>402 (71,9%)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>394 (74,6%)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>410 (73,7%)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>413 (74,4%)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>410 (70,8%)</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>430 (72,9%)</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>378 (75,6%)</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>328 (58,7%)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>344 (59,1%)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>289 (55,4%)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>317 (59,7%)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>319 (58,1%)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>298 (57,4%)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>327 (54,0%)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>332 (56,5%)</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>309 (56,8%)</t>
         </is>
       </c>
     </row>

</xml_diff>